<commit_message>
Update Excel sheet with latest data
</commit_message>
<xml_diff>
--- a/public/nConnect Module Status.xlsx
+++ b/public/nConnect Module Status.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ramji/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ramji/Documents/executive-dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C50F9DF8-1E2D-5045-AAF1-A1F655AA37A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F031A66-B7FA-1D49-B1B3-3099402D85F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="On Going" sheetId="2" r:id="rId1"/>
+    <sheet name="Ongoing" sheetId="2" r:id="rId1"/>
     <sheet name="Recently Deployed" sheetId="3" r:id="rId2"/>
-    <sheet name="Up Coming" sheetId="4" r:id="rId3"/>
+    <sheet name="Upcoming" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="124">
   <si>
     <t>Module Name</t>
   </si>
@@ -39,9 +39,6 @@
   </si>
   <si>
     <t>Branch Analytics</t>
-  </si>
-  <si>
-    <t>On Going</t>
   </si>
   <si>
     <t>Retention Calling</t>
@@ -132,9 +129,6 @@
     <t>Tags and Filter Issues</t>
   </si>
   <si>
-    <t xml:space="preserve">On Going </t>
-  </si>
-  <si>
     <t>Parent Check - in Module(Phase 2)</t>
   </si>
   <si>
@@ -153,12 +147,6 @@
   </si>
   <si>
     <t xml:space="preserve">user should be able to post as per student first language </t>
-  </si>
-  <si>
-    <t>nScribe enhancements phase2</t>
-  </si>
-  <si>
-    <t>House Keeping &amp; Security(Flutter)</t>
   </si>
   <si>
     <t>Branch &amp; Building Selection in Feedback Form
@@ -173,15 +161,9 @@
  Feedback Form – Submit Button Validation</t>
   </si>
   <si>
-    <t>House Keeping &amp; Security(BackEnd)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Replace Designation-Based Access with Permission-Based Access
  Update Daily Form Availability Window
  </t>
-  </si>
-  <si>
-    <t>House Keeping &amp; Security(Admin&amp;Web App)</t>
   </si>
   <si>
     <t>Branch Auth Tab in Admin Panel
@@ -311,13 +293,7 @@
     <t>HR Operations</t>
   </si>
   <si>
-    <t>UP Coming</t>
-  </si>
-  <si>
     <t>Module wise Analytics</t>
-  </si>
-  <si>
-    <t>Up Coming</t>
   </si>
   <si>
     <t>Adoption Calling (Revamp)</t>
@@ -526,12 +502,6 @@
     <t>Implementing Distance report and Daily report</t>
   </si>
   <si>
-    <t>Hierarchical heatmap/OLAP-style explorer
-An interactive view of Adoption Calling parent conversations, scored Month-Wise - click any state to drill into its branches, segments, and classes, with monthly movement colour-coded for instant scan.
-Isue Condensation
-Teacher Score</t>
-  </si>
-  <si>
     <t>Route Management - nTransport</t>
   </si>
   <si>
@@ -553,6 +523,52 @@
   </si>
   <si>
     <t>Concern grace period flow along auto closed concern</t>
+  </si>
+  <si>
+    <t>nScribe Enhancements phase2</t>
+  </si>
+  <si>
+    <t>Housekeeping &amp; Security Module</t>
+  </si>
+  <si>
+    <t>In the web app, after selecting the role, add an option to select the shift type as Day Shift or Night Shift.
+Introduce HKS Analytics sub-module under for analytics related to biometric and feedback forms.
+Add password visibility option for branches in the Branch Auth ID screen.</t>
+  </si>
+  <si>
+    <t>Adoption Calling Module</t>
+  </si>
+  <si>
+    <t>Enhancements planned for the Adoption Calling Staff App to make the module more actionable and insight driven using nScribe signals.
+Key focus areas:
+Student prioritisation
+Pre-call context for teachers
+Better visibility of important insights generated through nScribe
+Improved decision-making and follow-up tracking during adoption calls</t>
+  </si>
+  <si>
+    <t>Hierarchical heatmap/OLAP-style explorer
+An interactive view of Adoption Calling parent conversations, scored Month-Wise - click any state to drill into its branches, segments, and classes, with monthly movement colour-coded for instant scan.
+Issue Condensation
+Teacher Score</t>
+  </si>
+  <si>
+    <t>HouseKeeping &amp; Security(Flutter)</t>
+  </si>
+  <si>
+    <t>HouseKeeping &amp; Security(BackEnd)</t>
+  </si>
+  <si>
+    <t>HouseKeeping &amp; Security(Admin&amp;Web App)</t>
+  </si>
+  <si>
+    <t>Ongoing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ongoing </t>
+  </si>
+  <si>
+    <t>Upcoming</t>
   </si>
 </sst>
 </file>
@@ -936,7 +952,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1034,6 +1050,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1367,7 +1386,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>2</v>
@@ -1391,10 +1410,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -1412,13 +1431,13 @@
     </row>
     <row r="3" spans="1:16" ht="64" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -1436,13 +1455,13 @@
     </row>
     <row r="4" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>7</v>
-      </c>
       <c r="C4" s="3" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -1460,13 +1479,13 @@
     </row>
     <row r="5" spans="1:16" ht="208" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>9</v>
-      </c>
       <c r="C5" s="3" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -1484,13 +1503,13 @@
     </row>
     <row r="6" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="C6" s="3" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -1508,13 +1527,13 @@
     </row>
     <row r="7" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>13</v>
-      </c>
       <c r="C7" s="3" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1532,13 +1551,13 @@
     </row>
     <row r="8" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -1556,13 +1575,13 @@
     </row>
     <row r="9" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="C9" s="3" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -1580,13 +1599,13 @@
     </row>
     <row r="10" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
@@ -1604,13 +1623,13 @@
     </row>
     <row r="11" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>19</v>
-      </c>
       <c r="C11" s="3" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -1628,13 +1647,13 @@
     </row>
     <row r="12" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
@@ -1652,13 +1671,13 @@
     </row>
     <row r="13" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>22</v>
-      </c>
       <c r="C13" s="3" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
@@ -1676,13 +1695,13 @@
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>24</v>
-      </c>
       <c r="C14" s="2" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
@@ -1700,13 +1719,13 @@
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
@@ -1724,13 +1743,13 @@
     </row>
     <row r="16" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>26</v>
-      </c>
       <c r="C16" s="3" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
@@ -1748,13 +1767,13 @@
     </row>
     <row r="17" spans="1:16" ht="60" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
@@ -1772,13 +1791,13 @@
     </row>
     <row r="18" spans="1:16" ht="30" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B18" s="20" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
@@ -1796,13 +1815,13 @@
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A19" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="19" t="s">
-        <v>30</v>
-      </c>
       <c r="C19" s="2" t="s">
-        <v>31</v>
+        <v>122</v>
       </c>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
@@ -1820,13 +1839,13 @@
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A20" s="21" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="B20" s="22" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
@@ -1844,13 +1863,13 @@
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A21" s="21" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B21" s="22" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
@@ -1868,13 +1887,13 @@
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A22" s="22" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="B22" s="22" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
@@ -1892,13 +1911,13 @@
     </row>
     <row r="23" spans="1:16" ht="30" x14ac:dyDescent="0.2">
       <c r="A23" s="21" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
@@ -1916,13 +1935,13 @@
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A24" s="24" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B24" s="24" t="s">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
@@ -1940,13 +1959,13 @@
     </row>
     <row r="25" spans="1:16" ht="30" x14ac:dyDescent="0.2">
       <c r="A25" s="24" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
@@ -4507,7 +4526,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>2</v>
@@ -4515,13 +4534,13 @@
     </row>
     <row r="2" spans="1:16" ht="80" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="8" t="s">
-        <v>34</v>
-      </c>
       <c r="C2" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -4539,13 +4558,13 @@
     </row>
     <row r="3" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -4563,13 +4582,13 @@
     </row>
     <row r="4" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -4587,13 +4606,13 @@
     </row>
     <row r="5" spans="1:16" ht="96" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
-        <v>38</v>
+        <v>112</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -4611,13 +4630,13 @@
     </row>
     <row r="6" spans="1:16" ht="160" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
-        <v>39</v>
+        <v>118</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -4635,13 +4654,13 @@
     </row>
     <row r="7" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
-        <v>41</v>
+        <v>119</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -4659,13 +4678,13 @@
     </row>
     <row r="8" spans="1:16" ht="240" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
-        <v>43</v>
+        <v>120</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -4683,13 +4702,13 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -4707,13 +4726,13 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
@@ -4731,13 +4750,13 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -4755,13 +4774,13 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" s="15" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
@@ -4779,13 +4798,13 @@
     </row>
     <row r="13" spans="1:16" ht="105" x14ac:dyDescent="0.2">
       <c r="A13" s="15" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B13" s="29" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
@@ -4803,13 +4822,13 @@
     </row>
     <row r="14" spans="1:16" ht="60" x14ac:dyDescent="0.2">
       <c r="A14" s="9" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
@@ -4827,13 +4846,13 @@
     </row>
     <row r="15" spans="1:16" ht="15" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
@@ -4851,13 +4870,13 @@
     </row>
     <row r="16" spans="1:16" ht="15" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
@@ -4875,13 +4894,13 @@
     </row>
     <row r="17" spans="1:17" ht="15" x14ac:dyDescent="0.2">
       <c r="A17" s="9" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
@@ -4899,13 +4918,13 @@
     </row>
     <row r="18" spans="1:17" ht="30" x14ac:dyDescent="0.2">
       <c r="A18" s="9" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B18" s="20" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
@@ -4923,13 +4942,13 @@
     </row>
     <row r="19" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A19" s="9" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B19" s="30" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
@@ -4947,13 +4966,13 @@
     </row>
     <row r="20" spans="1:17" ht="30" x14ac:dyDescent="0.2">
       <c r="A20" s="9" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
@@ -4971,13 +4990,13 @@
     </row>
     <row r="21" spans="1:17" ht="15" x14ac:dyDescent="0.2">
       <c r="A21" s="9" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
@@ -4995,13 +5014,13 @@
     </row>
     <row r="22" spans="1:17" ht="15" x14ac:dyDescent="0.2">
       <c r="A22" s="9" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
@@ -5019,13 +5038,13 @@
     </row>
     <row r="23" spans="1:17" ht="45" x14ac:dyDescent="0.2">
       <c r="A23" s="9" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
@@ -5043,13 +5062,13 @@
     </row>
     <row r="24" spans="1:17" ht="15" x14ac:dyDescent="0.2">
       <c r="A24" s="9" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
@@ -5067,13 +5086,13 @@
     </row>
     <row r="25" spans="1:17" ht="30" x14ac:dyDescent="0.2">
       <c r="A25" s="9" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="B25" s="20" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
@@ -5091,13 +5110,13 @@
     </row>
     <row r="26" spans="1:17" ht="15" x14ac:dyDescent="0.2">
       <c r="A26" s="9" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
@@ -5115,13 +5134,13 @@
     </row>
     <row r="27" spans="1:17" ht="15" x14ac:dyDescent="0.2">
       <c r="A27" s="9" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
@@ -5139,13 +5158,13 @@
     </row>
     <row r="28" spans="1:17" ht="15" x14ac:dyDescent="0.2">
       <c r="A28" s="9" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
@@ -5163,13 +5182,13 @@
     </row>
     <row r="29" spans="1:17" ht="112" x14ac:dyDescent="0.2">
       <c r="A29" s="9" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D29" s="7"/>
       <c r="E29" s="1"/>
@@ -5187,13 +5206,13 @@
     </row>
     <row r="30" spans="1:17" ht="15" x14ac:dyDescent="0.2">
       <c r="A30" s="16" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="B30" s="17" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="C30" s="18" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D30" s="17"/>
       <c r="E30" s="1"/>
@@ -5212,13 +5231,13 @@
     </row>
     <row r="31" spans="1:17" ht="15" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
@@ -5237,13 +5256,13 @@
     </row>
     <row r="32" spans="1:17" ht="15" x14ac:dyDescent="0.2">
       <c r="A32" s="31" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D32" s="10"/>
       <c r="E32" s="10"/>
@@ -5262,13 +5281,13 @@
     </row>
     <row r="33" spans="1:17" ht="15" x14ac:dyDescent="0.2">
       <c r="A33" s="32" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D33" s="10"/>
       <c r="E33" s="10"/>
@@ -5315,7 +5334,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="32.796875" customWidth="1"/>
@@ -5337,57 +5356,79 @@
     </row>
     <row r="2" spans="1:3" ht="48" x14ac:dyDescent="0.2">
       <c r="A2" s="27" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B2" s="28" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="C2" s="27" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="45" x14ac:dyDescent="0.2">
       <c r="A3" s="27" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>80</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15" x14ac:dyDescent="0.2">
       <c r="A4" s="27" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="B4" s="27" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="C4" s="27" t="s">
-        <v>80</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="60" x14ac:dyDescent="0.2">
       <c r="A5" s="22" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>80</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="90" x14ac:dyDescent="0.2">
       <c r="A6" s="22" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="B6" s="23" t="s">
+        <v>117</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="45" x14ac:dyDescent="0.2">
+      <c r="A7" s="33" t="s">
+        <v>113</v>
+      </c>
+      <c r="B7" s="20" t="s">
         <v>114</v>
       </c>
-      <c r="C6" s="22" t="s">
-        <v>78</v>
+      <c r="C7" s="22" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="105" x14ac:dyDescent="0.2">
+      <c r="A8" s="33" t="s">
+        <v>115</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>116</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update nConnect Module Status excel sheet with latest data
</commit_message>
<xml_diff>
--- a/public/nConnect Module Status.xlsx
+++ b/public/nConnect Module Status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ramji/Documents/executive-dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F031A66-B7FA-1D49-B1B3-3099402D85F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{899E07E2-C9AC-F643-9C8C-09A9460C003B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="129">
   <si>
     <t>Module Name</t>
   </si>
@@ -531,11 +531,6 @@
     <t>Housekeeping &amp; Security Module</t>
   </si>
   <si>
-    <t>In the web app, after selecting the role, add an option to select the shift type as Day Shift or Night Shift.
-Introduce HKS Analytics sub-module under for analytics related to biometric and feedback forms.
-Add password visibility option for branches in the Branch Auth ID screen.</t>
-  </si>
-  <si>
     <t>Adoption Calling Module</t>
   </si>
   <si>
@@ -569,6 +564,25 @@
   </si>
   <si>
     <t>Upcoming</t>
+  </si>
+  <si>
+    <t>Service Desk Revamp</t>
+  </si>
+  <si>
+    <t>Adoption Calling- Staff App</t>
+  </si>
+  <si>
+    <t>Revamoping the module in UI and Migration</t>
+  </si>
+  <si>
+    <t>House Keeping</t>
+  </si>
+  <si>
+    <t>Add password visibility option for branches in the Branch Auth ID screen.</t>
+  </si>
+  <si>
+    <t>In the web app, after selecting the role, add an option to select the shift type as Day Shift or Night Shift.
+Introduce HKS Analytics sub-module under for analytics related to biometric and feedback forms.</t>
   </si>
 </sst>
 </file>
@@ -614,7 +628,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -641,8 +655,14 @@
         <fgColor rgb="FFB4C6E7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="23">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -948,11 +968,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF1F2329"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF1F2329"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1016,9 +1060,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1054,6 +1095,33 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1413,7 +1481,7 @@
         <v>76</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -1437,7 +1505,7 @@
         <v>77</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -1461,7 +1529,7 @@
         <v>6</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -1485,7 +1553,7 @@
         <v>8</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -1509,7 +1577,7 @@
         <v>10</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -1533,7 +1601,7 @@
         <v>12</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1557,7 +1625,7 @@
         <v>10</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -1581,7 +1649,7 @@
         <v>15</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -1605,7 +1673,7 @@
         <v>15</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
@@ -1629,7 +1697,7 @@
         <v>18</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -1653,7 +1721,7 @@
         <v>19</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
@@ -1677,7 +1745,7 @@
         <v>21</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
@@ -1701,7 +1769,7 @@
         <v>23</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
@@ -1725,7 +1793,7 @@
         <v>105</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
@@ -1749,7 +1817,7 @@
         <v>25</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
@@ -1773,7 +1841,7 @@
         <v>93</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
@@ -1797,7 +1865,7 @@
         <v>81</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
@@ -1821,7 +1889,7 @@
         <v>29</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
@@ -1838,14 +1906,14 @@
       <c r="P19" s="1"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="39" t="s">
         <v>79</v>
       </c>
-      <c r="B20" s="22" t="s">
+      <c r="B20" s="21" t="s">
         <v>80</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
@@ -1862,14 +1930,14 @@
       <c r="P20" s="1"/>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="39" t="s">
         <v>86</v>
       </c>
-      <c r="B21" s="22" t="s">
+      <c r="B21" s="21" t="s">
         <v>87</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
@@ -1886,14 +1954,14 @@
       <c r="P21" s="1"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A22" s="22" t="s">
+      <c r="A22" s="40" t="s">
         <v>88</v>
       </c>
-      <c r="B22" s="22" t="s">
+      <c r="B22" s="21" t="s">
         <v>89</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
@@ -1910,14 +1978,14 @@
       <c r="P22" s="1"/>
     </row>
     <row r="23" spans="1:16" ht="30" x14ac:dyDescent="0.2">
-      <c r="A23" s="21" t="s">
+      <c r="A23" s="39" t="s">
         <v>90</v>
       </c>
-      <c r="B23" s="23" t="s">
+      <c r="B23" s="22" t="s">
         <v>91</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
@@ -1934,14 +2002,14 @@
       <c r="P23" s="1"/>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A24" s="24" t="s">
+      <c r="A24" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="24" t="s">
+      <c r="B24" s="23" t="s">
         <v>111</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
@@ -1958,14 +2026,14 @@
       <c r="P24" s="1"/>
     </row>
     <row r="25" spans="1:16" ht="30" x14ac:dyDescent="0.2">
-      <c r="A25" s="24" t="s">
+      <c r="A25" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="B25" s="23" t="s">
+      <c r="B25" s="37" t="s">
         <v>92</v>
       </c>
-      <c r="C25" s="14" t="s">
-        <v>121</v>
+      <c r="C25" s="38" t="s">
+        <v>120</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
@@ -1982,9 +2050,15 @@
       <c r="P25" s="1"/>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
+      <c r="A26" s="23" t="s">
+        <v>123</v>
+      </c>
+      <c r="B26" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="C26" s="23" t="s">
+        <v>120</v>
+      </c>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
@@ -1999,10 +2073,16 @@
       <c r="O26" s="1"/>
       <c r="P26" s="1"/>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A27" s="1"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
+    <row r="27" spans="1:16" ht="105" x14ac:dyDescent="0.2">
+      <c r="A27" s="23" t="s">
+        <v>124</v>
+      </c>
+      <c r="B27" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="C27" s="23" t="s">
+        <v>120</v>
+      </c>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
@@ -2018,9 +2098,15 @@
       <c r="P27" s="1"/>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
+      <c r="A28" s="23" t="s">
+        <v>126</v>
+      </c>
+      <c r="B28" s="23" t="s">
+        <v>127</v>
+      </c>
+      <c r="C28" s="23" t="s">
+        <v>120</v>
+      </c>
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
@@ -2035,10 +2121,16 @@
       <c r="O28" s="1"/>
       <c r="P28" s="1"/>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A29" s="1"/>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
+    <row r="29" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+      <c r="A29" s="41" t="s">
+        <v>71</v>
+      </c>
+      <c r="B29" s="27" t="s">
+        <v>82</v>
+      </c>
+      <c r="C29" s="41" t="s">
+        <v>120</v>
+      </c>
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
@@ -2053,10 +2145,16 @@
       <c r="O29" s="1"/>
       <c r="P29" s="1"/>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A30" s="1"/>
-      <c r="B30" s="1"/>
-      <c r="C30" s="1"/>
+    <row r="30" spans="1:16" ht="45" x14ac:dyDescent="0.2">
+      <c r="A30" s="41" t="s">
+        <v>72</v>
+      </c>
+      <c r="B30" s="22" t="s">
+        <v>83</v>
+      </c>
+      <c r="C30" s="41" t="s">
+        <v>120</v>
+      </c>
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
@@ -4630,7 +4728,7 @@
     </row>
     <row r="6" spans="1:16" ht="160" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B6" s="8" t="s">
         <v>36</v>
@@ -4654,7 +4752,7 @@
     </row>
     <row r="7" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>37</v>
@@ -4678,7 +4776,7 @@
     </row>
     <row r="8" spans="1:16" ht="240" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B8" s="8" t="s">
         <v>38</v>
@@ -4800,7 +4898,7 @@
       <c r="A13" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="28" t="s">
         <v>46</v>
       </c>
       <c r="C13" s="14" t="s">
@@ -4944,7 +5042,7 @@
       <c r="A19" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="30" t="s">
+      <c r="B19" s="29" t="s">
         <v>103</v>
       </c>
       <c r="C19" s="7" t="s">
@@ -5255,7 +5353,7 @@
       <c r="Q31" s="10"/>
     </row>
     <row r="32" spans="1:17" ht="15" x14ac:dyDescent="0.2">
-      <c r="A32" s="31" t="s">
+      <c r="A32" s="30" t="s">
         <v>107</v>
       </c>
       <c r="B32" s="10" t="s">
@@ -5280,7 +5378,7 @@
       <c r="Q32" s="10"/>
     </row>
     <row r="33" spans="1:17" ht="15" x14ac:dyDescent="0.2">
-      <c r="A33" s="32" t="s">
+      <c r="A33" s="31" t="s">
         <v>106</v>
       </c>
       <c r="B33" s="10" t="s">
@@ -5334,7 +5432,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="32.796875" customWidth="1"/>
@@ -5344,91 +5442,69 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="25" t="s">
+      <c r="C1" s="24" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="48" x14ac:dyDescent="0.2">
-      <c r="A2" s="27" t="s">
-        <v>71</v>
-      </c>
-      <c r="B2" s="28" t="s">
-        <v>82</v>
-      </c>
-      <c r="C2" s="27" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="45" x14ac:dyDescent="0.2">
-      <c r="A3" s="27" t="s">
-        <v>72</v>
-      </c>
-      <c r="B3" s="23" t="s">
-        <v>83</v>
-      </c>
-      <c r="C3" s="27" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="15" x14ac:dyDescent="0.2">
-      <c r="A4" s="27" t="s">
+    <row r="2" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A2" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="B4" s="27" t="s">
+      <c r="B2" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="C4" s="27" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="60" x14ac:dyDescent="0.2">
-      <c r="A5" s="22" t="s">
+      <c r="C2" s="26" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="60" x14ac:dyDescent="0.2">
+      <c r="A3" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="B5" s="23" t="s">
+      <c r="B3" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="C5" s="27" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="90" x14ac:dyDescent="0.2">
-      <c r="A6" s="22" t="s">
+      <c r="C3" s="26" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="90" x14ac:dyDescent="0.2">
+      <c r="A4" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="B6" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="C6" s="22" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="45" x14ac:dyDescent="0.2">
-      <c r="A7" s="33" t="s">
+      <c r="B4" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="30" x14ac:dyDescent="0.2">
+      <c r="A5" s="32" t="s">
         <v>113</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="B5" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="105" x14ac:dyDescent="0.2">
+      <c r="A6" s="33" t="s">
         <v>114</v>
       </c>
-      <c r="C7" s="22" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="105" x14ac:dyDescent="0.2">
-      <c r="A8" s="33" t="s">
+      <c r="B6" s="34" t="s">
         <v>115</v>
       </c>
-      <c r="B8" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="C8" s="22" t="s">
-        <v>123</v>
+      <c r="C6" s="35" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>